<commit_message>
Diagnose each export before coding it; fix multi-select columns
Labelling real answers surfaced three problems the pipeline hid:

- a 1,654-row "why did you buy?" column was a multi-select pick-list being
  coded as free text, inflating counts and theme shares for that brand
- the shared codebook could not place ~30% of answers for some brands
- two exports pasted side by side were treated as one question

Adds `voc diagnose` (question kinds, coverage gaps, pasted exports, candidate
vocabulary, draft keyword file), multi-select detection and per-option
tallying, industry keyword packs, and codebook v2.2 with first_time_trial,
loyalty_rewards and site_usability. Labelling kits now offer `unclear` plus a
note, and `voc eval` reports those rows as a coverage gap instead of scoring
them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/output/demo_apparel_pdp_poll_report.xlsx
+++ b/examples/output/demo_apparel_pdp_poll_report.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1045" uniqueCount="147">
   <si>
     <t>Field</t>
   </si>
@@ -75,10 +75,10 @@
     <t>-</t>
   </si>
   <si>
-    <t>2.0.1</t>
-  </si>
-  <si>
-    <t>2026-09-17T09:35:38</t>
+    <t>2.2</t>
+  </si>
+  <si>
+    <t>2026-09-17T11:50:15</t>
   </si>
   <si>
     <t>Identifying columns (names, emails, locations, IPs, order ids) were removed at ingest. Spend is shown only as a band. Emails, phones, URLs and handles inside answers are masked.</t>
@@ -144,6 +144,9 @@
     <t>quality</t>
   </si>
   <si>
+    <t>site_usability</t>
+  </si>
+  <si>
     <t>design_style</t>
   </si>
   <si>
@@ -174,6 +177,9 @@
     <t>Quality &amp; durability</t>
   </si>
   <si>
+    <t>Site &amp; buying experience</t>
+  </si>
+  <si>
     <t>Design &amp; style</t>
   </si>
   <si>
@@ -237,6 +243,9 @@
     <t>stock_availability;repeat_loyalty</t>
   </si>
   <si>
+    <t>site_usability;payment_checkout</t>
+  </si>
+  <si>
     <t>stock_availability;size_fit</t>
   </si>
   <si>
@@ -288,6 +297,12 @@
     <t>no_concern</t>
   </si>
   <si>
+    <t>first_time_trial</t>
+  </si>
+  <si>
+    <t>loyalty_rewards</t>
+  </si>
+  <si>
     <t>Efficacy &amp; results</t>
   </si>
   <si>
@@ -315,6 +330,12 @@
     <t>Nothing / no concern</t>
   </si>
   <si>
+    <t>First-time trial</t>
+  </si>
+  <si>
+    <t>Loyalty &amp; rewards</t>
+  </si>
+  <si>
     <t>Precio y valor</t>
   </si>
   <si>
@@ -369,6 +390,15 @@
     <t>Ninguna / sin inquietud</t>
   </si>
   <si>
+    <t>Primera compra / probar la marca</t>
+  </si>
+  <si>
+    <t>Lealtad y recompensas</t>
+  </si>
+  <si>
+    <t>Experiencia de compra en el sitio</t>
+  </si>
+  <si>
     <t>Price, discounts, promotions, or value for money.</t>
   </si>
   <si>
@@ -421,6 +451,15 @@
   </si>
   <si>
     <t>The customer explicitly had no concern or nothing to add.</t>
+  </si>
+  <si>
+    <t>Curiosity or trying the brand for the first time, with no prior experience of it.</t>
+  </si>
+  <si>
+    <t>Loyalty points, rewards, referral credit, memberships, subscriptions.</t>
+  </si>
+  <si>
+    <t>How easy the store itself is to use: finding things, the size selector, the cart, errors, unclear labels or steps.</t>
   </si>
 </sst>
 </file>
@@ -537,9 +576,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Themes!$D$2:$D$11</c:f>
+              <c:f>Themes!$D$2:$D$12</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>Size &amp; fit</c:v>
                 </c:pt>
@@ -568,6 +607,9 @@
                   <c:v>Quality &amp; durability</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>Site &amp; buying experience</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>Design &amp; style</c:v>
                 </c:pt>
               </c:strCache>
@@ -575,10 +617,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Themes!$H$2:$H$11</c:f>
+              <c:f>Themes!$H$2:$H$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>0.3083333333333333</c:v>
                 </c:pt>
@@ -607,6 +649,9 @@
                   <c:v>0.025</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>0.01666666666666667</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>0.008333333333333333</c:v>
                 </c:pt>
               </c:numCache>
@@ -665,8 +710,8 @@
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1099,13 +1144,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="26.7109375" customWidth="1"/>
     <col min="5" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" style="4" customWidth="1"/>
     <col min="9" max="9" width="12.7109375" customWidth="1"/>
@@ -1151,7 +1195,7 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2">
         <v>37</v>
@@ -1180,7 +1224,7 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3">
         <v>29</v>
@@ -1209,7 +1253,7 @@
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4">
         <v>16</v>
@@ -1238,7 +1282,7 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5">
         <v>15</v>
@@ -1267,13 +1311,13 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E6">
         <v>14</v>
       </c>
       <c r="F6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G6">
         <v>120</v>
@@ -1296,7 +1340,7 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -1325,7 +1369,7 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -1354,7 +1398,7 @@
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9">
         <v>5</v>
@@ -1383,7 +1427,7 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -1412,21 +1456,50 @@
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11">
         <v>120</v>
       </c>
       <c r="H11" s="4">
+        <v>0.01666666666666667</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>120</v>
+      </c>
+      <c r="H12" s="4">
         <v>0.008333333333333333</v>
       </c>
-      <c r="I11" t="b">
+      <c r="I12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1452,13 +1525,13 @@
         <v>21</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>29</v>
@@ -1466,7 +1539,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B2">
         <v>900</v>
@@ -1488,21 +1561,21 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>36</v>
@@ -1517,15 +1590,18 @@
         <v>33</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:10">
       <c r="A2" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1546,15 +1622,18 @@
         <v>12</v>
       </c>
       <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
         <v>6</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1575,15 +1654,18 @@
         <v>4</v>
       </c>
       <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
         <v>8</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1592,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -1604,15 +1686,18 @@
         <v>5</v>
       </c>
       <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
         <v>7</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:10">
       <c r="A5" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1621,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1633,15 +1718,18 @@
         <v>4</v>
       </c>
       <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>4</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:10">
       <c r="A6" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1662,9 +1750,12 @@
         <v>1</v>
       </c>
       <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>9</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>3</v>
       </c>
     </row>
@@ -1690,7 +1781,7 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>21</v>
@@ -1699,22 +1790,22 @@
         <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1728,10 +1819,10 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F2" t="s">
         <v>33</v>
@@ -1740,10 +1831,10 @@
         <v>33</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1757,7 +1848,7 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F3" t="s">
         <v>33</v>
@@ -1766,10 +1857,10 @@
         <v>33</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1783,7 +1874,7 @@
         <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
         <v>32</v>
@@ -1792,10 +1883,10 @@
         <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1809,7 +1900,7 @@
         <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
         <v>32</v>
@@ -1818,10 +1909,10 @@
         <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1835,7 +1926,7 @@
         <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
         <v>32</v>
@@ -1844,10 +1935,10 @@
         <v>32</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1861,7 +1952,7 @@
         <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
         <v>40</v>
@@ -1870,10 +1961,10 @@
         <v>40</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1887,7 +1978,7 @@
         <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F8" t="s">
         <v>32</v>
@@ -1896,10 +1987,10 @@
         <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1913,7 +2004,7 @@
         <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F9" t="s">
         <v>35</v>
@@ -1922,10 +2013,10 @@
         <v>35</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I9" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1939,7 +2030,7 @@
         <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
         <v>38</v>
@@ -1948,10 +2039,10 @@
         <v>38</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1965,7 +2056,7 @@
         <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
         <v>36</v>
@@ -1974,10 +2065,10 @@
         <v>36</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1991,7 +2082,7 @@
         <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F12" t="s">
         <v>33</v>
@@ -2000,10 +2091,10 @@
         <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2017,19 +2108,19 @@
         <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F13" t="s">
         <v>37</v>
       </c>
       <c r="G13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2043,7 +2134,7 @@
         <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F14" t="s">
         <v>33</v>
@@ -2052,10 +2143,10 @@
         <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I14" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2069,7 +2160,7 @@
         <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F15" t="s">
         <v>33</v>
@@ -2078,10 +2169,10 @@
         <v>33</v>
       </c>
       <c r="H15" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -2095,7 +2186,7 @@
         <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F16" t="s">
         <v>33</v>
@@ -2104,10 +2195,10 @@
         <v>33</v>
       </c>
       <c r="H16" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -2121,7 +2212,7 @@
         <v>31</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
         <v>32</v>
@@ -2130,10 +2221,10 @@
         <v>32</v>
       </c>
       <c r="H17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I17" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -2147,19 +2238,19 @@
         <v>31</v>
       </c>
       <c r="D18" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F18" t="s">
         <v>34</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I18" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -2173,7 +2264,7 @@
         <v>31</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F19" t="s">
         <v>35</v>
@@ -2182,10 +2273,10 @@
         <v>35</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I19" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -2199,7 +2290,7 @@
         <v>31</v>
       </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
         <v>32</v>
@@ -2208,10 +2299,10 @@
         <v>32</v>
       </c>
       <c r="H20" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I20" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -2225,7 +2316,7 @@
         <v>31</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
         <v>33</v>
@@ -2234,10 +2325,10 @@
         <v>33</v>
       </c>
       <c r="H21" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I21" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -2251,7 +2342,7 @@
         <v>31</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F22" t="s">
         <v>36</v>
@@ -2260,10 +2351,10 @@
         <v>36</v>
       </c>
       <c r="H22" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I22" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -2277,7 +2368,7 @@
         <v>31</v>
       </c>
       <c r="D23" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F23" t="s">
         <v>36</v>
@@ -2286,10 +2377,10 @@
         <v>36</v>
       </c>
       <c r="H23" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I23" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -2303,7 +2394,7 @@
         <v>31</v>
       </c>
       <c r="D24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F24" t="s">
         <v>34</v>
@@ -2312,10 +2403,10 @@
         <v>34</v>
       </c>
       <c r="H24" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I24" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -2329,19 +2420,19 @@
         <v>31</v>
       </c>
       <c r="D25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F25" t="s">
         <v>34</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H25" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I25" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -2355,19 +2446,19 @@
         <v>31</v>
       </c>
       <c r="D26" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F26" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G26" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="H26" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I26" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -2381,7 +2472,7 @@
         <v>31</v>
       </c>
       <c r="D27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F27" t="s">
         <v>34</v>
@@ -2390,10 +2481,10 @@
         <v>34</v>
       </c>
       <c r="H27" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I27" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -2407,7 +2498,7 @@
         <v>31</v>
       </c>
       <c r="D28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F28" t="s">
         <v>34</v>
@@ -2416,10 +2507,10 @@
         <v>34</v>
       </c>
       <c r="H28" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I28" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -2433,7 +2524,7 @@
         <v>31</v>
       </c>
       <c r="D29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F29" t="s">
         <v>32</v>
@@ -2442,10 +2533,10 @@
         <v>32</v>
       </c>
       <c r="H29" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I29" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -2459,7 +2550,7 @@
         <v>31</v>
       </c>
       <c r="D30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F30" t="s">
         <v>34</v>
@@ -2468,10 +2559,10 @@
         <v>34</v>
       </c>
       <c r="H30" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I30" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -2485,7 +2576,7 @@
         <v>31</v>
       </c>
       <c r="D31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F31" t="s">
         <v>33</v>
@@ -2494,10 +2585,10 @@
         <v>33</v>
       </c>
       <c r="H31" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I31" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -2511,7 +2602,7 @@
         <v>31</v>
       </c>
       <c r="D32" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F32" t="s">
         <v>32</v>
@@ -2520,10 +2611,10 @@
         <v>32</v>
       </c>
       <c r="H32" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I32" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2537,19 +2628,19 @@
         <v>31</v>
       </c>
       <c r="D33" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F33" t="s">
         <v>34</v>
       </c>
       <c r="G33" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H33" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I33" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2563,7 +2654,7 @@
         <v>31</v>
       </c>
       <c r="D34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F34" t="s">
         <v>34</v>
@@ -2572,10 +2663,10 @@
         <v>34</v>
       </c>
       <c r="H34" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I34" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2589,19 +2680,19 @@
         <v>31</v>
       </c>
       <c r="D35" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F35" t="s">
         <v>34</v>
       </c>
       <c r="G35" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H35" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I35" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2615,7 +2706,7 @@
         <v>31</v>
       </c>
       <c r="D36" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F36" t="s">
         <v>34</v>
@@ -2624,10 +2715,10 @@
         <v>34</v>
       </c>
       <c r="H36" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I36" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2641,19 +2732,19 @@
         <v>31</v>
       </c>
       <c r="D37" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F37" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G37" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H37" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I37" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2667,7 +2758,7 @@
         <v>31</v>
       </c>
       <c r="D38" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F38" t="s">
         <v>33</v>
@@ -2676,10 +2767,10 @@
         <v>33</v>
       </c>
       <c r="H38" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I38" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2693,7 +2784,7 @@
         <v>31</v>
       </c>
       <c r="D39" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F39" t="s">
         <v>35</v>
@@ -2702,10 +2793,10 @@
         <v>35</v>
       </c>
       <c r="H39" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I39" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2719,19 +2810,19 @@
         <v>31</v>
       </c>
       <c r="D40" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F40" t="s">
         <v>34</v>
       </c>
       <c r="G40" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H40" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I40" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2745,10 +2836,10 @@
         <v>31</v>
       </c>
       <c r="D41" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E41" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F41" t="s">
         <v>32</v>
@@ -2757,10 +2848,10 @@
         <v>32</v>
       </c>
       <c r="H41" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I41" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2774,7 +2865,7 @@
         <v>31</v>
       </c>
       <c r="D42" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F42" t="s">
         <v>33</v>
@@ -2783,10 +2874,10 @@
         <v>33</v>
       </c>
       <c r="H42" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I42" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2800,7 +2891,7 @@
         <v>31</v>
       </c>
       <c r="D43" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F43" t="s">
         <v>32</v>
@@ -2809,10 +2900,10 @@
         <v>32</v>
       </c>
       <c r="H43" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I43" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2826,7 +2917,7 @@
         <v>31</v>
       </c>
       <c r="D44" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F44" t="s">
         <v>35</v>
@@ -2835,10 +2926,10 @@
         <v>35</v>
       </c>
       <c r="H44" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I44" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2852,7 +2943,7 @@
         <v>31</v>
       </c>
       <c r="D45" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F45" t="s">
         <v>33</v>
@@ -2861,10 +2952,10 @@
         <v>33</v>
       </c>
       <c r="H45" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I45" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2878,7 +2969,7 @@
         <v>31</v>
       </c>
       <c r="D46" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F46" t="s">
         <v>33</v>
@@ -2887,10 +2978,10 @@
         <v>33</v>
       </c>
       <c r="H46" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I46" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2904,7 +2995,7 @@
         <v>31</v>
       </c>
       <c r="D47" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F47" t="s">
         <v>35</v>
@@ -2913,10 +3004,10 @@
         <v>35</v>
       </c>
       <c r="H47" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I47" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2930,7 +3021,7 @@
         <v>31</v>
       </c>
       <c r="D48" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F48" t="s">
         <v>36</v>
@@ -2939,10 +3030,10 @@
         <v>36</v>
       </c>
       <c r="H48" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I48" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2956,7 +3047,7 @@
         <v>31</v>
       </c>
       <c r="D49" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F49" t="s">
         <v>40</v>
@@ -2965,10 +3056,10 @@
         <v>40</v>
       </c>
       <c r="H49" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I49" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2982,7 +3073,7 @@
         <v>31</v>
       </c>
       <c r="D50" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F50" t="s">
         <v>33</v>
@@ -2991,10 +3082,10 @@
         <v>33</v>
       </c>
       <c r="H50" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I50" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -3008,19 +3099,19 @@
         <v>31</v>
       </c>
       <c r="D51" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F51" t="s">
         <v>34</v>
       </c>
       <c r="G51" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H51" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I51" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -3034,7 +3125,7 @@
         <v>31</v>
       </c>
       <c r="D52" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F52" t="s">
         <v>33</v>
@@ -3043,10 +3134,10 @@
         <v>33</v>
       </c>
       <c r="H52" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I52" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -3060,7 +3151,7 @@
         <v>31</v>
       </c>
       <c r="D53" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F53" t="s">
         <v>32</v>
@@ -3069,10 +3160,10 @@
         <v>32</v>
       </c>
       <c r="H53" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I53" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -3086,7 +3177,7 @@
         <v>31</v>
       </c>
       <c r="D54" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F54" t="s">
         <v>33</v>
@@ -3095,10 +3186,10 @@
         <v>33</v>
       </c>
       <c r="H54" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I54" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -3112,7 +3203,7 @@
         <v>31</v>
       </c>
       <c r="D55" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F55" t="s">
         <v>32</v>
@@ -3121,10 +3212,10 @@
         <v>32</v>
       </c>
       <c r="H55" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I55" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -3138,7 +3229,7 @@
         <v>31</v>
       </c>
       <c r="D56" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F56" t="s">
         <v>36</v>
@@ -3147,10 +3238,10 @@
         <v>36</v>
       </c>
       <c r="H56" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I56" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -3164,7 +3255,7 @@
         <v>31</v>
       </c>
       <c r="D57" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F57" t="s">
         <v>35</v>
@@ -3173,10 +3264,10 @@
         <v>35</v>
       </c>
       <c r="H57" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I57" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -3190,10 +3281,10 @@
         <v>31</v>
       </c>
       <c r="D58" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E58" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F58" t="s">
         <v>38</v>
@@ -3202,10 +3293,10 @@
         <v>38</v>
       </c>
       <c r="H58" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I58" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -3219,7 +3310,7 @@
         <v>31</v>
       </c>
       <c r="D59" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F59" t="s">
         <v>32</v>
@@ -3228,10 +3319,10 @@
         <v>32</v>
       </c>
       <c r="H59" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I59" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -3245,7 +3336,7 @@
         <v>31</v>
       </c>
       <c r="D60" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F60" t="s">
         <v>36</v>
@@ -3254,10 +3345,10 @@
         <v>36</v>
       </c>
       <c r="H60" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I60" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -3271,7 +3362,7 @@
         <v>31</v>
       </c>
       <c r="D61" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F61" t="s">
         <v>34</v>
@@ -3280,10 +3371,10 @@
         <v>34</v>
       </c>
       <c r="H61" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I61" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -3297,7 +3388,7 @@
         <v>31</v>
       </c>
       <c r="D62" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F62" t="s">
         <v>32</v>
@@ -3306,10 +3397,10 @@
         <v>32</v>
       </c>
       <c r="H62" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I62" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -3323,7 +3414,7 @@
         <v>31</v>
       </c>
       <c r="D63" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F63" t="s">
         <v>33</v>
@@ -3332,10 +3423,10 @@
         <v>33</v>
       </c>
       <c r="H63" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I63" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -3349,7 +3440,7 @@
         <v>31</v>
       </c>
       <c r="D64" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F64" t="s">
         <v>35</v>
@@ -3358,10 +3449,10 @@
         <v>35</v>
       </c>
       <c r="H64" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I64" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -3375,7 +3466,7 @@
         <v>31</v>
       </c>
       <c r="D65" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F65" t="s">
         <v>36</v>
@@ -3384,10 +3475,10 @@
         <v>36</v>
       </c>
       <c r="H65" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I65" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -3401,7 +3492,7 @@
         <v>31</v>
       </c>
       <c r="D66" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F66" t="s">
         <v>32</v>
@@ -3410,10 +3501,10 @@
         <v>32</v>
       </c>
       <c r="H66" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I66" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -3427,19 +3518,19 @@
         <v>31</v>
       </c>
       <c r="D67" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F67" t="s">
         <v>37</v>
       </c>
       <c r="G67" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H67" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I67" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -3453,7 +3544,7 @@
         <v>31</v>
       </c>
       <c r="D68" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F68" t="s">
         <v>35</v>
@@ -3462,10 +3553,10 @@
         <v>35</v>
       </c>
       <c r="H68" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I68" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3479,7 +3570,7 @@
         <v>31</v>
       </c>
       <c r="D69" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F69" t="s">
         <v>33</v>
@@ -3488,10 +3579,10 @@
         <v>33</v>
       </c>
       <c r="H69" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I69" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3505,7 +3596,7 @@
         <v>31</v>
       </c>
       <c r="D70" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F70" t="s">
         <v>32</v>
@@ -3514,10 +3605,10 @@
         <v>32</v>
       </c>
       <c r="H70" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I70" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3531,7 +3622,7 @@
         <v>31</v>
       </c>
       <c r="D71" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F71" t="s">
         <v>38</v>
@@ -3540,10 +3631,10 @@
         <v>38</v>
       </c>
       <c r="H71" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I71" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3557,7 +3648,7 @@
         <v>31</v>
       </c>
       <c r="D72" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F72" t="s">
         <v>37</v>
@@ -3566,10 +3657,10 @@
         <v>37</v>
       </c>
       <c r="H72" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I72" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3583,7 +3674,7 @@
         <v>31</v>
       </c>
       <c r="D73" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F73" t="s">
         <v>32</v>
@@ -3592,10 +3683,10 @@
         <v>32</v>
       </c>
       <c r="H73" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I73" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3609,7 +3700,7 @@
         <v>31</v>
       </c>
       <c r="D74" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F74" t="s">
         <v>32</v>
@@ -3618,10 +3709,10 @@
         <v>32</v>
       </c>
       <c r="H74" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I74" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3635,7 +3726,7 @@
         <v>31</v>
       </c>
       <c r="D75" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F75" t="s">
         <v>35</v>
@@ -3644,10 +3735,10 @@
         <v>35</v>
       </c>
       <c r="H75" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I75" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3661,7 +3752,7 @@
         <v>31</v>
       </c>
       <c r="D76" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F76" t="s">
         <v>38</v>
@@ -3670,10 +3761,10 @@
         <v>38</v>
       </c>
       <c r="H76" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I76" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3687,19 +3778,19 @@
         <v>31</v>
       </c>
       <c r="D77" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F77" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G77" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="H77" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I77" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3713,7 +3804,7 @@
         <v>31</v>
       </c>
       <c r="D78" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F78" t="s">
         <v>33</v>
@@ -3722,10 +3813,10 @@
         <v>33</v>
       </c>
       <c r="H78" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I78" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3739,7 +3830,7 @@
         <v>31</v>
       </c>
       <c r="D79" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F79" t="s">
         <v>33</v>
@@ -3748,10 +3839,10 @@
         <v>33</v>
       </c>
       <c r="H79" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I79" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3765,19 +3856,19 @@
         <v>31</v>
       </c>
       <c r="D80" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F80" t="s">
         <v>34</v>
       </c>
       <c r="G80" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H80" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I80" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3791,10 +3882,10 @@
         <v>31</v>
       </c>
       <c r="D81" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E81" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F81" t="s">
         <v>32</v>
@@ -3803,10 +3894,10 @@
         <v>32</v>
       </c>
       <c r="H81" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I81" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3820,7 +3911,7 @@
         <v>31</v>
       </c>
       <c r="D82" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F82" t="s">
         <v>33</v>
@@ -3829,10 +3920,10 @@
         <v>33</v>
       </c>
       <c r="H82" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I82" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3846,7 +3937,7 @@
         <v>31</v>
       </c>
       <c r="D83" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F83" t="s">
         <v>40</v>
@@ -3855,10 +3946,10 @@
         <v>40</v>
       </c>
       <c r="H83" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I83" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -3872,7 +3963,7 @@
         <v>31</v>
       </c>
       <c r="D84" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F84" t="s">
         <v>33</v>
@@ -3881,10 +3972,10 @@
         <v>33</v>
       </c>
       <c r="H84" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I84" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -3898,7 +3989,7 @@
         <v>31</v>
       </c>
       <c r="D85" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F85" t="s">
         <v>36</v>
@@ -3907,10 +3998,10 @@
         <v>36</v>
       </c>
       <c r="H85" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I85" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -3924,7 +4015,7 @@
         <v>31</v>
       </c>
       <c r="D86" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F86" t="s">
         <v>33</v>
@@ -3933,10 +4024,10 @@
         <v>33</v>
       </c>
       <c r="H86" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I86" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -3950,7 +4041,7 @@
         <v>31</v>
       </c>
       <c r="D87" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F87" t="s">
         <v>35</v>
@@ -3959,10 +4050,10 @@
         <v>35</v>
       </c>
       <c r="H87" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I87" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -3976,7 +4067,7 @@
         <v>31</v>
       </c>
       <c r="D88" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F88" t="s">
         <v>32</v>
@@ -3985,10 +4076,10 @@
         <v>32</v>
       </c>
       <c r="H88" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I88" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -4002,7 +4093,7 @@
         <v>31</v>
       </c>
       <c r="D89" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F89" t="s">
         <v>32</v>
@@ -4011,10 +4102,10 @@
         <v>32</v>
       </c>
       <c r="H89" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I89" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -4028,7 +4119,7 @@
         <v>31</v>
       </c>
       <c r="D90" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F90" t="s">
         <v>38</v>
@@ -4037,10 +4128,10 @@
         <v>38</v>
       </c>
       <c r="H90" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I90" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -4054,7 +4145,7 @@
         <v>31</v>
       </c>
       <c r="D91" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F91" t="s">
         <v>35</v>
@@ -4063,10 +4154,10 @@
         <v>35</v>
       </c>
       <c r="H91" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I91" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -4080,7 +4171,7 @@
         <v>31</v>
       </c>
       <c r="D92" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F92" t="s">
         <v>32</v>
@@ -4089,10 +4180,10 @@
         <v>32</v>
       </c>
       <c r="H92" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I92" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -4106,7 +4197,7 @@
         <v>31</v>
       </c>
       <c r="D93" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F93" t="s">
         <v>36</v>
@@ -4115,10 +4206,10 @@
         <v>36</v>
       </c>
       <c r="H93" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I93" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -4132,7 +4223,7 @@
         <v>31</v>
       </c>
       <c r="D94" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F94" t="s">
         <v>36</v>
@@ -4141,10 +4232,10 @@
         <v>36</v>
       </c>
       <c r="H94" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I94" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -4158,7 +4249,7 @@
         <v>31</v>
       </c>
       <c r="D95" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F95" t="s">
         <v>33</v>
@@ -4167,10 +4258,10 @@
         <v>33</v>
       </c>
       <c r="H95" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I95" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -4184,7 +4275,7 @@
         <v>31</v>
       </c>
       <c r="D96" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F96" t="s">
         <v>35</v>
@@ -4193,10 +4284,10 @@
         <v>35</v>
       </c>
       <c r="H96" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I96" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -4210,7 +4301,7 @@
         <v>31</v>
       </c>
       <c r="D97" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F97" t="s">
         <v>37</v>
@@ -4219,10 +4310,10 @@
         <v>37</v>
       </c>
       <c r="H97" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I97" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -4236,7 +4327,7 @@
         <v>31</v>
       </c>
       <c r="D98" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F98" t="s">
         <v>32</v>
@@ -4245,10 +4336,10 @@
         <v>32</v>
       </c>
       <c r="H98" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I98" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -4262,7 +4353,7 @@
         <v>31</v>
       </c>
       <c r="D99" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F99" t="s">
         <v>32</v>
@@ -4271,10 +4362,10 @@
         <v>32</v>
       </c>
       <c r="H99" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I99" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -4288,7 +4379,7 @@
         <v>31</v>
       </c>
       <c r="D100" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F100" t="s">
         <v>35</v>
@@ -4297,10 +4388,10 @@
         <v>35</v>
       </c>
       <c r="H100" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I100" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -4314,10 +4405,10 @@
         <v>31</v>
       </c>
       <c r="D101" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E101" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F101" t="s">
         <v>33</v>
@@ -4326,10 +4417,10 @@
         <v>33</v>
       </c>
       <c r="H101" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I101" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -4343,7 +4434,7 @@
         <v>31</v>
       </c>
       <c r="D102" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F102" t="s">
         <v>32</v>
@@ -4352,10 +4443,10 @@
         <v>32</v>
       </c>
       <c r="H102" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I102" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -4369,19 +4460,19 @@
         <v>31</v>
       </c>
       <c r="D103" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F103" t="s">
         <v>37</v>
       </c>
       <c r="G103" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H103" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I103" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -4395,7 +4486,7 @@
         <v>31</v>
       </c>
       <c r="D104" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F104" t="s">
         <v>33</v>
@@ -4404,10 +4495,10 @@
         <v>33</v>
       </c>
       <c r="H104" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I104" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -4421,7 +4512,7 @@
         <v>31</v>
       </c>
       <c r="D105" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F105" t="s">
         <v>35</v>
@@ -4430,10 +4521,10 @@
         <v>35</v>
       </c>
       <c r="H105" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I105" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -4447,7 +4538,7 @@
         <v>31</v>
       </c>
       <c r="D106" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F106" t="s">
         <v>32</v>
@@ -4456,10 +4547,10 @@
         <v>32</v>
       </c>
       <c r="H106" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I106" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -4473,7 +4564,7 @@
         <v>31</v>
       </c>
       <c r="D107" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F107" t="s">
         <v>33</v>
@@ -4482,10 +4573,10 @@
         <v>33</v>
       </c>
       <c r="H107" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I107" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -4499,7 +4590,7 @@
         <v>31</v>
       </c>
       <c r="D108" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F108" t="s">
         <v>32</v>
@@ -4508,10 +4599,10 @@
         <v>32</v>
       </c>
       <c r="H108" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I108" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -4525,7 +4616,7 @@
         <v>31</v>
       </c>
       <c r="D109" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F109" t="s">
         <v>32</v>
@@ -4534,10 +4625,10 @@
         <v>32</v>
       </c>
       <c r="H109" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I109" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -4551,7 +4642,7 @@
         <v>31</v>
       </c>
       <c r="D110" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F110" t="s">
         <v>35</v>
@@ -4560,10 +4651,10 @@
         <v>35</v>
       </c>
       <c r="H110" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I110" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -4577,7 +4668,7 @@
         <v>31</v>
       </c>
       <c r="D111" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F111" t="s">
         <v>37</v>
@@ -4586,10 +4677,10 @@
         <v>37</v>
       </c>
       <c r="H111" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I111" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -4603,7 +4694,7 @@
         <v>31</v>
       </c>
       <c r="D112" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F112" t="s">
         <v>32</v>
@@ -4612,10 +4703,10 @@
         <v>32</v>
       </c>
       <c r="H112" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I112" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -4629,7 +4720,7 @@
         <v>31</v>
       </c>
       <c r="D113" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F113" t="s">
         <v>32</v>
@@ -4638,10 +4729,10 @@
         <v>32</v>
       </c>
       <c r="H113" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I113" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -4655,7 +4746,7 @@
         <v>31</v>
       </c>
       <c r="D114" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F114" t="s">
         <v>36</v>
@@ -4664,10 +4755,10 @@
         <v>36</v>
       </c>
       <c r="H114" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I114" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -4681,7 +4772,7 @@
         <v>31</v>
       </c>
       <c r="D115" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F115" t="s">
         <v>34</v>
@@ -4690,10 +4781,10 @@
         <v>34</v>
       </c>
       <c r="H115" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I115" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -4707,7 +4798,7 @@
         <v>31</v>
       </c>
       <c r="D116" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F116" t="s">
         <v>32</v>
@@ -4716,10 +4807,10 @@
         <v>32</v>
       </c>
       <c r="H116" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I116" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -4733,7 +4824,7 @@
         <v>31</v>
       </c>
       <c r="D117" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F117" t="s">
         <v>32</v>
@@ -4742,10 +4833,10 @@
         <v>32</v>
       </c>
       <c r="H117" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I117" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -4759,7 +4850,7 @@
         <v>31</v>
       </c>
       <c r="D118" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F118" t="s">
         <v>32</v>
@@ -4768,10 +4859,10 @@
         <v>32</v>
       </c>
       <c r="H118" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I118" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -4785,7 +4876,7 @@
         <v>31</v>
       </c>
       <c r="D119" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F119" t="s">
         <v>36</v>
@@ -4794,10 +4885,10 @@
         <v>36</v>
       </c>
       <c r="H119" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I119" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -4811,19 +4902,19 @@
         <v>31</v>
       </c>
       <c r="D120" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F120" t="s">
         <v>34</v>
       </c>
       <c r="G120" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H120" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I120" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -4837,7 +4928,7 @@
         <v>31</v>
       </c>
       <c r="D121" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F121" t="s">
         <v>32</v>
@@ -4846,10 +4937,10 @@
         <v>32</v>
       </c>
       <c r="H121" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I121" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -4863,10 +4954,10 @@
         <v>31</v>
       </c>
       <c r="D122" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E122" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F122" t="s">
         <v>35</v>
@@ -4875,10 +4966,10 @@
         <v>35</v>
       </c>
       <c r="H122" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I122" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -4888,27 +4979,27 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="27.7109375" customWidth="1"/>
-    <col min="3" max="3" width="29.7109375" customWidth="1"/>
-    <col min="4" max="4" width="71.7109375" customWidth="1"/>
+    <col min="3" max="3" width="35.7109375" customWidth="1"/>
+    <col min="4" max="4" width="80.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4916,13 +5007,13 @@
         <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -4930,55 +5021,55 @@
         <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C6" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D6" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -4986,13 +5077,13 @@
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -5000,13 +5091,13 @@
         <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D8" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -5014,13 +5105,13 @@
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -5028,83 +5119,83 @@
         <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D10" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C11" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="D12" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D14" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D15" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -5112,27 +5203,27 @@
         <v>38</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D16" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D17" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -5140,27 +5231,69 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D18" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
-        <v>133</v>
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D21" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D22" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>